<commit_message>
feat: implement GitLab CI/CD pipeline and add comprehensive documentation for testing, building, and deployment
</commit_message>
<xml_diff>
--- a/docs/AxiaOps_Phase2_TaskTracking.xlsx
+++ b/docs/AxiaOps_Phase2_TaskTracking.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,8 +67,41 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00C00000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="0000B050"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00FFC000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000070C0"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +138,12 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070AD47"/>
+        <bgColor rgb="0070AD47"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -157,6 +196,22 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -522,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -536,9 +591,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AxiaOps Phase 2 (Alpha) — Task Tracking</t>
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>AxiaOps Phase 2 (Alpha) — Task Tracking | Updated: April 11, 2026 — 3:00 PM</t>
         </is>
       </c>
     </row>
@@ -577,7 +632,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Implemented slog/Sentry/Prometheus | Tests: logging_test.go (output formats, log levels)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -619,7 +674,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Implemented with slog, Sentry SDK, Prometheus metrics</t>
+          <t>All /v1/ routes, nginx proxy configured | Tests: handler_test.go (/v1/ prefix verification)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -661,7 +716,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>All routes use /v1/ format; nginx proxy configured</t>
+          <t>Per-tenant sliding window, 60 req/min | Tests: ratelimit_test.go (isolation, token bucket, concurrent access)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -678,12 +733,12 @@
     <row r="7" ht="40" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>✅ Rate Limiting (In-memory token bucket)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>DONE</t>
+          <t>✅ Graceful Shutdown (SIGTERM handling)</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>✅ DONE</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -703,7 +758,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Per-tenant sliding window, 60 req/min; disabled in DEV_MODE</t>
+          <t>signal.NotifyContext + server.Shutdown() in API &amp; ingestion services. 30-sec timeout, request draining, DB cleanup. Test: make test-shutdown</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1127,6 +1182,90 @@
       <c r="A27" t="inlineStr">
         <is>
           <t>July 2026: Production deployment to App Runner + RDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>NEXT STEPS &amp; DEPENDENCIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>🎯 PRIORITY: Graceful Shutdown (P0, May 1 target)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Blocker for: Scheduled Auto-Scan, Redis Integration, Production Deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>🔧 GRACEFUL SHUTDOWN IMPLEMENTATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>API Service (services/api/cmd/main.go, lines 200-243):</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓ signal.NotifyContext(shutdownCtx, os.Interrupt, syscall.SIGTERM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓ server.Shutdown(shutdownCtx) with 30-second timeout</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓ Request draining, database cleanup, logging</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="23" t="inlineStr">
+        <is>
+          <t>Ingestion Service (services/ingestion/cmd/main.go, lines 167-210):</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓ Same pattern: signal.NotifyContext + server.Shutdown()</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✓ Handles both SIGTERM (App Runner) and SIGINT (Ctrl+C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="24" t="inlineStr">
+        <is>
+          <t>📝 Test Command: make test-shutdown</t>
         </is>
       </c>
     </row>

</xml_diff>